<commit_message>
Final changes made with tested experimental results file
</commit_message>
<xml_diff>
--- a/artifacts/Experimental_results.xlsx
+++ b/artifacts/Experimental_results.xlsx
@@ -19,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +49,54 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00444444"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000D652D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -71,8 +118,28 @@
         <fgColor rgb="00FFF4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -94,11 +161,25 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +205,44 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,1393 +608,1307 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:N60"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
-    <col width="70" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="3" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="C1" s="1" t="inlineStr">
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Project:</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Same Table / 糖友同枱 - shared home dinner planning for diabetes patients (Hospital Authority, classroom prototype)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>There are three pipelines in this app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Pipeline 1 (understand the cook's request) is highly relevant to the project objective and therefore, it requires finetuning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Pipeline 2 (retrieve dishes from the labeled library) does not require finetuning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Pipeline 3 (turn a Cantonese voice note into the request text) does not require finetuning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Experiment: Selecting the optimal model(s)</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Experiment: Assessing the overall performance</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>Step 1: Select THREE relevant and comparable pre-trained models</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>Step 2a: Finetune the selected models with own dataset</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="inlineStr">
-        <is>
-          <t>Step 3: Implement the App and deploy it to Streamlit Cloud</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Pipeline 1 - Multi-label text classification (to be finetuned)</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Fine-tuning</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>1. Deployment</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Dataset:</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>data/train/p1_train.jsonl, p1_eval.jsonl, p1_test.jsonl</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>App = pipeline 1 (finetuned hfl/chinese-roberta-wwm-ext) + pipeline 2 (BAAI/bge-small-zh-v1.5, hybrid weight 3) + plating rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>training samples:</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>3000</v>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Pipeline 1 as deployed (finetuned model + keyword lexicon), accuracy on the hand-written sentences: 0.852</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>evaluation samples:</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>testing samples (hand-written):</t>
-        </is>
-      </c>
-      <c r="F13" s="3">
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Same Table / 糖友同枱 — shared home dinner planning for diabetes patients</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Three pipelines: P1 text-classification (finetuned) · P2 dish retrieval (embeddings) · P3 Cantonese ASR (not finetuned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>BLOCK A — Pipeline 1 (multi-label text classification)</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>BLOCK B — Pipeline 2 (feature extraction / retrieval)</t>
+        </is>
+      </c>
+      <c r="M4" s="22" t="inlineStr">
+        <is>
+          <t>BLOCK C — App tests (20 requests) + Voice (5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>p1_train / p1_eval / p1_test.jsonl</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>3000 / 600 /</t>
+        </is>
+      </c>
+      <c r="D5" s="23">
         <f>COUNTA('P1 test'!A2:A109)</f>
         <v/>
       </c>
-      <c r="J13" s="1" t="inlineStr">
-        <is>
-          <t>2. Test and evaluate the App (20 test samples)</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Objective judgement: tags, dish count, no repeats, methods, soup, 20-min, balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Inputs (people | request | chips)</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Outputs (tags found | menu)</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>Correct or not (notebook)</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>Checked on Streamlit Cloud (fill in: Correct / Incorrect)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>hand-written</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>p2_dev / p2_test + paraphrase / library</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="J5" s="23">
+        <f>COUNTA('P2 queries'!A2:A201)</f>
+        <v/>
+      </c>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>24 para / 100 dishes</t>
+        </is>
+      </c>
+      <c r="M5" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="N5" s="24" t="inlineStr">
+        <is>
+          <t>Query (people | request)</t>
+        </is>
+      </c>
+      <c r="O5" s="24" t="inlineStr">
+        <is>
+          <t>Expected tags</t>
+        </is>
+      </c>
+      <c r="P5" s="24" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="Q5" s="24" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Accuracy (after finetuning, using trainer.evaluate())</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Run time (in sec. per 100 requests, CPU)</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Fine-tuning time (in sec.)</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Accuracy on hand-written test</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 1</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Eval accuracy</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>Runtime s/100</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Hand-test acc</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>Model name</t>
+        </is>
+      </c>
+      <c r="I6" s="24" t="inlineStr">
+        <is>
+          <t>Top-5 (literal)</t>
+        </is>
+      </c>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>Runtime s/100</t>
+        </is>
+      </c>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>Top-1 accuracy</t>
+        </is>
+      </c>
+      <c r="M6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="26" t="inlineStr">
         <is>
           <t>4 people | 阿爸牙唔好，想食啲軟熟嘅蒸餸，唔好太甜</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>tags: less_sweet, steam | 不會失敗的蒸蛋 / 清蒸山藥｜三鮮肉丸 / 蝦仁蒸蛋豆腐 / 甜豌豆炒菇 / 蒜炒小白菜/快炒/5分鐘/簡單快速 / 客家鹹湯圓的“炒料”</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="O6" s="26" t="inlineStr">
+        <is>
+          <t>less_sweet, steam</t>
+        </is>
+      </c>
+      <c r="P6" s="27" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="N15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="62" customHeight="1">
-      <c r="C16" s="5" t="inlineStr">
+      <c r="Q6" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Model 1</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>hfl/rbt3</t>
         </is>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="C7" s="28" t="n">
         <v>0.595</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="D7" s="25" t="n">
         <v>2.97</v>
       </c>
-      <c r="G16" s="10" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="H16" s="8" t="n">
+      <c r="E7" s="28" t="n">
         <v>0.8148</v>
       </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 2</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="G7" s="27" t="inlineStr">
+        <is>
+          <t>Model 1</t>
+        </is>
+      </c>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>BAAI/bge-small-zh-v1.5</t>
+        </is>
+      </c>
+      <c r="I7" s="30">
+        <f>COUNTIF('P2 queries'!D2:D201,"&lt;=5")/COUNT('P2 queries'!D2:D201)</f>
+        <v/>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K7" s="30">
+        <f>COUNTIF('P2 queries'!D2:D201,1)/COUNT('P2 queries'!D2:D201)</f>
+        <v/>
+      </c>
+      <c r="M7" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="26" t="inlineStr">
         <is>
           <t>2 people | 今晚好趕，求其炒兩個餸就算</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>tags: quick, stir | 好市多牛三寶炒蒜苗 / 菠菜炒鴻禧菇 / 蒜炒小白菜/快炒/5分鐘/簡單快速</t>
-        </is>
-      </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="O7" s="26" t="inlineStr">
+        <is>
+          <t>quick, stir</t>
+        </is>
+      </c>
+      <c r="P7" s="27" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="N16" s="7" t="n"/>
-    </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="C17" s="5" t="inlineStr">
+      <c r="Q7" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Model 2</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>hfl/rbt6</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="C8" s="28" t="n">
         <v>0.6032999999999999</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="D8" s="25" t="n">
         <v>5.44</v>
       </c>
-      <c r="G17" s="10" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="H17" s="8" t="n">
+      <c r="E8" s="28" t="n">
         <v>0.8611</v>
       </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 3</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>Model 2</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>shibing624/text2vec-base-chinese</t>
+        </is>
+      </c>
+      <c r="I8" s="28">
+        <f>COUNTIF('P2 queries'!E2:E201,"&lt;=5")/COUNT('P2 queries'!E2:E201)</f>
+        <v/>
+      </c>
+      <c r="J8" s="25" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K8" s="28">
+        <f>COUNTIF('P2 queries'!E2:E201,1)/COUNT('P2 queries'!E2:E201)</f>
+        <v/>
+      </c>
+      <c r="M8" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="26" t="inlineStr">
         <is>
           <t>6 people | 想煲湯，另外加個白灼菜</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>tags: blanch, soup | 白切雞 / 『涼拌皮蛋』－清爽、酸辣、開胃。 / 涼拌魚皮 / 芹菜炒花枝 / 家常小菜-涼拌干絲 / 《料理簡單做》涼拌萵筍/菜心 / 涼拌萵筍 ( A菜心 ) / 客家鹹湯圓的“炒料”</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="O8" s="26" t="inlineStr">
+        <is>
+          <t>blanch, soup</t>
+        </is>
+      </c>
+      <c r="P8" s="27" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="N17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="62" customHeight="1">
-      <c r="C18" s="11" t="inlineStr">
+      <c r="Q8" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Model 3</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>hfl/chinese-roberta-wwm-ext</t>
         </is>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="C9" s="30" t="n">
         <v>0.6667</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="D9" s="27" t="n">
         <v>10.78</v>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="H18" s="12">
+      <c r="E9" s="30">
         <f>COUNTIF('P1 test'!D2:D109,"Correct")/COUNTA('P1 test'!D2:D109)</f>
         <v/>
       </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 4</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>5 people | 屋企有三個男仔，肉要多</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="inlineStr">
-        <is>
-          <t>tags: more_meat | 好市多牛三寶炒蒜苗 / 十三香炒回鍋肉 / 青椒炒肉絲 - 家常料理 / 菠菜炒鴻禧菇 / 免炒無油無糖自製棗泥 / 素食版的粄條😋 蔬炒粄條🤤 / 薑絲石斑魚蛤蜊湯</t>
-        </is>
-      </c>
-      <c r="M18" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="62" customHeight="1">
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>keyword lexicon (no model, no training)</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>0.3983</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8" t="n">
-        <v>0.6481</v>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 5</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
-          <t>3 people | 最近食得好油，想清清地</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
-        <is>
-          <t>tags: more_veg | 『涼拌皮蛋』－清爽、酸辣、開胃。 / 清炒小黃瓜 / 蒜炒菜心 / 山藥排骨湯</t>
-        </is>
-      </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N19" s="7" t="n"/>
-    </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>MoritzLaurer/mDeBERTa-v3-base-mnli-xnli (zero-shot, no training)</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>2371.15</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="8" t="n">
-        <v>0.287</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 6</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>4 people | (empty box)  [chips: steam, soup]</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>tags: soup, steam | 不會失敗的蒸蛋 / 清蒸山藥｜三鮮肉丸 / 清蒸石斑魚 / 百合蒸东星斑 / 炒結頭菜乾 / 🍲懶人火鍋_康寶極湯味日式高湯包</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="n"/>
-    </row>
-    <row r="21" ht="62" customHeight="1">
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>Accuracy = all 8 tags of a sentence correct (exact match). Settings: 3 epochs, learning rate 5e-05, batch 16, fine-tuned on cuda. Source: notebooks/Model1_finetune_tagger.ipynb. The picked model's hand-written accuracy is a formula over sheet 'P1 test'.</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 7</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>4 people | (empty box)</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>tags: (none) | 青椒炒肉絲 - 家常料理 / 好市多牛三寶炒蒜苗 / 蒜香鮮蝦炒彩蔬 / 家常小菜-涼拌干絲 / 《料理簡單做》涼拌萵筍/菜心 / 客家鹹湯圓的“炒料”</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N21" s="7" t="n"/>
-    </row>
-    <row r="22" ht="62" customHeight="1">
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 8</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>1 people | 七點先放工，要十五分鐘搞得掂</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
-        <is>
-          <t>tags: quick | 十三香炒回鍋肉 / 蒜炒小白菜/快炒/5分鐘/簡單快速</t>
-        </is>
-      </c>
-      <c r="M22" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="62" customHeight="1">
-      <c r="E23" s="1" t="inlineStr">
-        <is>
-          <t>Step 2b: Pick the BEST finetuned model for implementation</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 9</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>6 people | 婆婆糖尿，醬汁唔可以甜  [chips: more_veg]</t>
-        </is>
-      </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>tags: less_sweet, more_veg | 好市多牛三寶炒蒜苗 / 炒櫻桃鴨胸 / 蝦仁炒毛豆 / 甜豌豆炒菇 / 涼拌櫛瓜 / 蒜炒菜心 / 薑絲高麗菜炒小黃瓜 / 白菜蛋花湯</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="n"/>
-    </row>
-    <row r="24" ht="62" customHeight="1">
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>hfl/chinese-roberta-wwm-ext is picked: highest evaluation accuracy; models within one standard error of the best are tied and the shortest run time wins.</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 10</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>3 people | 今晚想吃清蒸的，配一個燙青菜</t>
-        </is>
-      </c>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>tags: blanch, steam | 清蒸山藥｜三鮮肉丸 / 清蒸石斑魚 / 家常小菜-涼拌干絲 / 榭黃芥菜羹｜立春節氣料理</t>
-        </is>
-      </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N24" s="7" t="n"/>
-    </row>
-    <row r="25" ht="62" customHeight="1">
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>The finetuned model is uploaded to Hugging Face as Tannedfish95/same-table-tagger and is used for implementing the App.</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 11</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>4 people | quick stir fry with lots of veggies</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>tags: more_veg, quick, stir | 爆香麻辣雞肝 / 芹菜炒花枝 / 薑絲高麗菜炒小黃瓜 / 芹菜小黃瓜炒豆腐 / 清炒小芥菜 / 酸菜豬血湯</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N25" s="7" t="n"/>
-    </row>
-    <row r="26" ht="62" customHeight="1">
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 12</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="inlineStr">
-        <is>
-          <t>5 people | we want more meat tonight and a soup</t>
-        </is>
-      </c>
-      <c r="L26" s="6" t="inlineStr">
-        <is>
-          <t>tags: more_veg, soup | 涼拌小黃瓜雞絲 / 芥藍菜炒鹹豬肉 / 蒜蓉蒸蝦 / 小黃瓜炒杏鮑菇及火腿片 / 清炒小芥菜 / 鹽炒花生 / 酸菜豬血湯</t>
-        </is>
-      </c>
-      <c r="M26" s="6" t="inlineStr">
-        <is>
-          <t>Incorrect (tags)</t>
-        </is>
-      </c>
-      <c r="N26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="62" customHeight="1">
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 13</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>2 people | 落雨天想飲啖熱湯</t>
-        </is>
-      </c>
-      <c r="L27" s="6" t="inlineStr">
-        <is>
-          <t>tags: soup | 豬肉辣炒高麗菜乾 / 涼拌萵筍 ( A菜心 ) / 🍲懶人火鍋_康寶極湯味日式高湯包</t>
-        </is>
-      </c>
-      <c r="M27" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N27" s="7" t="n"/>
-    </row>
-    <row r="28" ht="62" customHeight="1">
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>Step 1: Select THREE relevant and comparable pre-trained models</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>Step 2a: Test the performance of the selected models with your own dataset</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 14</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>4 people | 想食得有鑊氣，炒牛肉都好</t>
-        </is>
-      </c>
-      <c r="L28" s="6" t="inlineStr">
-        <is>
-          <t>tags: stir | 好市多牛三寶炒蒜苗 / 香菇肉末炒龍鬚菜 / 洋蔥毛肚炒蒜苗 / 清炒小黃瓜 / 芹菜鮮蔬炒豆乾 / 清燉牛肉湯</t>
-        </is>
-      </c>
-      <c r="M28" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N28" s="7" t="n"/>
-    </row>
-    <row r="29" ht="62" customHeight="1">
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>Pipeline 2 - Feature extraction (sentence embeddings for dish retrieval, not finetuned)</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 15</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="inlineStr">
-        <is>
-          <t>6 people | 蒸魚，炒菜，再加個湯</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>tags: soup, steam, stir | 不會失敗的蒸蛋 / 清蒸山藥｜三鮮肉丸 / 懶人蒸爐料理-鳳梨醬蒸魚 / 清蒸石斑魚 / 蒜炒小白菜/快炒/5分鐘/簡單快速 / 百合蒸东星斑 / 炒結頭菜乾 / 客家鹹湯圓的“炒料”</t>
-        </is>
-      </c>
-      <c r="M29" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N29" s="7" t="n"/>
-    </row>
-    <row r="30" ht="62" customHeight="1">
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Dataset:</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>data/train/p2_dev.jsonl (development), p2_test.jsonl + p2_paraphrase_test.jsonl (testing)</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 16</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr">
-        <is>
-          <t>3 people | 十五分鐘煮好，灼個菜蒸條魚</t>
-        </is>
-      </c>
-      <c r="L30" s="6" t="inlineStr">
-        <is>
-          <t>tags: blanch, quick, steam | 不會失敗的蒸蛋 / 懶人蒸爐料理-鳳梨醬蒸魚 / 蒜炒小白菜/快炒/5分鐘/簡單快速 / 薑絲石斑魚蛤蜊湯</t>
-        </is>
-      </c>
-      <c r="M30" s="6" t="inlineStr">
-        <is>
-          <t>Incorrect (methods on menu)</t>
-        </is>
-      </c>
-      <c r="N30" s="7" t="n"/>
-    </row>
-    <row r="31" ht="62" customHeight="1">
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>development samples (set the hybrid weight):</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 17</t>
-        </is>
-      </c>
-      <c r="K31" s="6" t="inlineStr">
-        <is>
-          <t>4 people | 多菜少肉，唔好甜  [chips: quick]</t>
-        </is>
-      </c>
-      <c r="L31" s="6" t="inlineStr">
-        <is>
-          <t>tags: less_sweet, more_veg, quick | 好市多牛三寶炒蒜苗 / 蝦仁炒毛豆 / 甜豌豆炒菇 / 薑絲高麗菜炒小黃瓜 / 蒜炒小白菜/快炒/5分鐘/簡單快速 / 鹹菜蒜頭蛤蠣雞湯（電鍋/一鍋到底）</t>
-        </is>
-      </c>
-      <c r="M31" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N31" s="7" t="n"/>
-    </row>
-    <row r="32" ht="62" customHeight="1">
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>testing samples (literal queries):</t>
-        </is>
-      </c>
-      <c r="F32" s="3">
-        <f>COUNTA('P2 queries'!A2:A201)</f>
-        <v/>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 18</t>
-        </is>
-      </c>
-      <c r="K32" s="6" t="inlineStr">
-        <is>
-          <t>2 people | 隨便啦  [chips: blanch]</t>
-        </is>
-      </c>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>tags: blanch | 白切雞 / 涼拌魚皮 / 家常小菜-涼拌干絲</t>
-        </is>
-      </c>
-      <c r="M32" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N32" s="7" t="n"/>
-    </row>
-    <row r="33" ht="62" customHeight="1">
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>testing samples (paraphrase queries):</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 19</t>
-        </is>
-      </c>
-      <c r="K33" s="6" t="inlineStr">
-        <is>
-          <t>5 people | 長輩血糖高，不要甜的</t>
-        </is>
-      </c>
-      <c r="L33" s="6" t="inlineStr">
-        <is>
-          <t>tags: less_sweet | 豬肉辣炒高麗菜乾 / 洋蔥炒鹹豬肉 / 蝦仁炒毛豆 / 古早味鯖魚罐頭炒高麗菜 / 甜豌豆炒菇 / 免炒無油無糖自製棗泥 / 酸菜豬血湯</t>
-        </is>
-      </c>
-      <c r="M33" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N33" s="7" t="n"/>
-    </row>
-    <row r="34" ht="62" customHeight="1">
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>library dishes searched:</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Test sample 20</t>
-        </is>
-      </c>
-      <c r="K34" s="6" t="inlineStr">
-        <is>
-          <t>4 people | 雪櫃有雞胸同菠菜</t>
-        </is>
-      </c>
-      <c r="L34" s="6" t="inlineStr">
-        <is>
-          <t>tags: (none) | 涼拌小黃瓜雞絲 / 炒櫻桃鴨胸 / 菠菜炒鴻禧菇 / 小黃瓜炒杏鮑菇 / 小黃瓜炒杏鮑菇及火腿片 / 鹹菜蒜頭蛤蠣雞湯（電鍋/一鍋到底）</t>
-        </is>
-      </c>
-      <c r="M34" s="6" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="N34" s="7" t="n"/>
-    </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Model name</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Performance (top-5 accuracy, literal queries)</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Run time (in sec. per 100 queries, CPU)</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Top-1 accuracy</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Paraphrase precision@5</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Hybrid weight w</t>
-        </is>
-      </c>
-      <c r="L36" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy (notebook):</t>
-        </is>
-      </c>
-      <c r="M36" s="3">
-        <f>COUNTIF(M15:M34,"Correct")&amp;" out of "&amp;COUNTA(M15:M34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>Model 1</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>BAAI/bge-small-zh-v1.5</t>
-        </is>
-      </c>
-      <c r="E37" s="12">
-        <f>COUNTIF('P2 queries'!D2:D201,"&lt;=5")/COUNT('P2 queries'!D2:D201)</f>
-        <v/>
-      </c>
-      <c r="F37" s="13" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G37" s="12">
-        <f>COUNTIF('P2 queries'!D2:D201,1)/COUNT('P2 queries'!D2:D201)</f>
-        <v/>
-      </c>
-      <c r="H37" s="12" t="n">
-        <v>0.5417</v>
-      </c>
-      <c r="I37" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="M37" s="16">
-        <f>COUNTIF(M15:M34,"Correct")/COUNTA(M15:M34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Model 2</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>shibing624/text2vec-base-chinese</t>
-        </is>
-      </c>
-      <c r="E38" s="8">
-        <f>COUNTIF('P2 queries'!E2:E201,"&lt;=5")/COUNT('P2 queries'!E2:E201)</f>
-        <v/>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="G38" s="8">
-        <f>COUNTIF('P2 queries'!E2:E201,1)/COUNT('P2 queries'!E2:E201)</f>
-        <v/>
-      </c>
-      <c r="H38" s="8" t="n">
-        <v>0.5833</v>
-      </c>
-      <c r="I38" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L38" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy (Streamlit Cloud):</t>
-        </is>
-      </c>
-      <c r="N38" s="16">
-        <f>IF(COUNTA(N15:N34)=0,"not checked yet",COUNTIF(N15:N34,"Correct")/COUNTA(N15:N34))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="C39" s="5" t="inlineStr">
+      <c r="G9" s="25" t="inlineStr">
         <is>
           <t>Model 3</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>sentence-transformers/paraphrase-multilingual-MiniLM-L12-v2</t>
-        </is>
-      </c>
-      <c r="E39" s="8">
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>paraphrase-multilingual-MiniLM-L12-v2</t>
+        </is>
+      </c>
+      <c r="I9" s="28">
         <f>COUNTIF('P2 queries'!F2:F201,"&lt;=5")/COUNT('P2 queries'!F2:F201)</f>
         <v/>
       </c>
-      <c r="F39" s="9" t="n">
+      <c r="J9" s="25" t="n">
         <v>1.04</v>
       </c>
-      <c r="G39" s="8">
+      <c r="K9" s="28">
         <f>COUNTIF('P2 queries'!F2:F201,1)/COUNT('P2 queries'!F2:F201)</f>
         <v/>
       </c>
-      <c r="H39" s="8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="C40" s="5" t="inlineStr">
+      <c r="M9" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="26" t="inlineStr">
+        <is>
+          <t>5 people | 屋企有三個男仔，肉要多</t>
+        </is>
+      </c>
+      <c r="O9" s="26" t="inlineStr">
+        <is>
+          <t>more_meat</t>
+        </is>
+      </c>
+      <c r="P9" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q9" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>keyword lexicon (no model)</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>0.3983</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E10" s="28" t="n">
+        <v>0.6481</v>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
         <is>
           <t>character TF-IDF (no model)</t>
         </is>
       </c>
-      <c r="E40" s="8">
+      <c r="I10" s="28">
         <f>COUNTIF('P2 queries'!C2:C201,"&lt;=5")/COUNT('P2 queries'!C2:C201)</f>
         <v/>
       </c>
-      <c r="F40" s="9" t="n">
+      <c r="J10" s="25" t="n">
         <v>0.24</v>
       </c>
-      <c r="G40" s="8">
+      <c r="K10" s="28">
         <f>COUNTIF('P2 queries'!C2:C201,1)/COUNT('P2 queries'!C2:C201)</f>
         <v/>
       </c>
-      <c r="H40" s="8" t="n">
-        <v>0.475</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr">
-        <is>
-          <t>Legend: fill the shaded column N after repeating each request on the deployed app (type Correct or Incorrect). Green rows = picked models.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="44" customHeight="1">
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>A query is correct when its target dish is ranked in the top 5 of the library (the menu shows 6-8 dishes). Each encoder runs through the app's Retriever: score = cosine similarity + w x character TF-IDF, with w set on the development queries only. Source: notebooks/Model2_experiments.ipynb; accuracy cells are formulas over sheet 'P2 queries'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="E43" s="1" t="inlineStr">
-        <is>
-          <t>Step 2b: Pick the BEST model for implementation</t>
-        </is>
-      </c>
-      <c r="J43" s="1" t="inlineStr">
-        <is>
-          <t>3. Voice-note tests on Streamlit Cloud (pipeline 3: alvanlii/whisper-small-cantonese)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>BAAI/bge-small-zh-v1.5 is picked: highest top-5 accuracy; models within one standard error of the best are tied and the shortest run time wins.</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>Say this into the app (Cantonese)</t>
-        </is>
-      </c>
-      <c r="L44" s="4" t="inlineStr">
-        <is>
-          <t>Expected tags</t>
-        </is>
-      </c>
-      <c r="M44" s="4" t="inlineStr">
-        <is>
-          <t>Text heard (fill in)</t>
-        </is>
-      </c>
-      <c r="N44" s="4" t="inlineStr">
-        <is>
-          <t>Correct or not (fill in)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="J45" s="5" t="inlineStr">
-        <is>
-          <t>Voice test 1</t>
-        </is>
-      </c>
-      <c r="K45" s="5" t="inlineStr">
-        <is>
-          <t>今晚想食清蒸魚，唔好太甜</t>
-        </is>
-      </c>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t>steam, less_sweet</t>
-        </is>
-      </c>
-      <c r="M45" s="7" t="n"/>
-      <c r="N45" s="7" t="n"/>
-    </row>
-    <row r="46">
-      <c r="J46" s="5" t="inlineStr">
-        <is>
-          <t>Voice test 2</t>
-        </is>
-      </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>好趕時間，炒兩個餸就得</t>
-        </is>
-      </c>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>quick, stir</t>
-        </is>
-      </c>
-      <c r="M46" s="7" t="n"/>
-      <c r="N46" s="7" t="n"/>
-    </row>
-    <row r="47">
-      <c r="C47" s="1" t="inlineStr">
-        <is>
-          <t>Step 1: Select THREE relevant and comparable pre-trained models</t>
-        </is>
-      </c>
-      <c r="E47" s="1" t="inlineStr">
-        <is>
-          <t>Step 2a: Test the performance of the selected models with your own dataset</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>Voice test 3</t>
-        </is>
-      </c>
-      <c r="K47" s="5" t="inlineStr">
-        <is>
-          <t>想煲個湯，多啲菜</t>
-        </is>
-      </c>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>soup, more_veg</t>
-        </is>
-      </c>
-      <c r="M47" s="7" t="n"/>
-      <c r="N47" s="7" t="n"/>
-    </row>
-    <row r="48">
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>Pipeline 3 - Automatic speech recognition (Cantonese voice notes, not finetuned)</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr">
-        <is>
-          <t>Voice test 4</t>
-        </is>
-      </c>
-      <c r="K48" s="5" t="inlineStr">
-        <is>
-          <t>屋企三個男仔，肉要多啲</t>
-        </is>
-      </c>
-      <c r="L48" s="5" t="inlineStr">
-        <is>
-          <t>more_meat</t>
-        </is>
-      </c>
-      <c r="M48" s="7" t="n"/>
-      <c r="N48" s="7" t="n"/>
-    </row>
-    <row r="49">
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Dataset:</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>data/speech/ (Mozilla Common Voice 22, Cantonese test split, CC0)</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>Voice test 5</t>
-        </is>
-      </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>灼個菜心，再蒸個水蛋</t>
-        </is>
-      </c>
-      <c r="L49" s="5" t="inlineStr">
+      <c r="M10" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="26" t="inlineStr">
+        <is>
+          <t>3 people | 最近食得好油，想清清地</t>
+        </is>
+      </c>
+      <c r="O10" s="26" t="inlineStr">
+        <is>
+          <t>more_veg</t>
+        </is>
+      </c>
+      <c r="P10" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q10" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>mDeBERTa-v3-base-mnli-xnli (zero-shot)</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>2371.15</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Para P@5</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>bge=0.5417 (w=3) · text2vec=0.5833 (w=2) · MiniLM=0.6 (w=5) · TF-IDF=0.475</t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="26" t="inlineStr">
+        <is>
+          <t>4 people | (empty box)  [chips: steam, soup]</t>
+        </is>
+      </c>
+      <c r="O11" s="26" t="inlineStr">
+        <is>
+          <t>soup, steam</t>
+        </is>
+      </c>
+      <c r="P11" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q11" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Exact-match on all 8 tags. 3 epochs, lr 5e-5, batch 16, cuda. FT times (s): rbt3=16.6, rbt6=27.6, roberta=54.2. Source: Model1_finetune_tagger.ipynb</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>Correct if target dish in top-5. score = cosine + w×TF-IDF (w on dev only). Col K = Top-1. Source: Model2_experiments.ipynb</t>
+        </is>
+      </c>
+      <c r="M12" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" s="26" t="inlineStr">
+        <is>
+          <t>4 people | (empty box)</t>
+        </is>
+      </c>
+      <c r="O12" s="26" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="P12" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q12" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>PICK</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>hfl/chinese-roberta-wwm-ext (highest eval acc). HF: Tannedfish95/same-table-tagger</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
+      <c r="G13" s="31" t="inlineStr">
+        <is>
+          <t>PICK</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>BAAI/bge-small-zh-v1.5 (highest top-5; hybrid w=3)</t>
+        </is>
+      </c>
+      <c r="I13" s="32" t="n"/>
+      <c r="J13" s="32" t="n"/>
+      <c r="K13" s="32" t="n"/>
+      <c r="M13" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" s="26" t="inlineStr">
+        <is>
+          <t>1 people | 七點先放工，要十五分鐘搞得掂</t>
+        </is>
+      </c>
+      <c r="O13" s="26" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="P13" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q13" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="M14" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="N14" s="26" t="inlineStr">
+        <is>
+          <t>6 people | 婆婆糖尿，醬汁唔可以甜  [chips: more_veg]</t>
+        </is>
+      </c>
+      <c r="O14" s="26" t="inlineStr">
+        <is>
+          <t>less_sweet, more_veg</t>
+        </is>
+      </c>
+      <c r="P14" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q14" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Pipeline 3 — ASR (Cantonese, not finetuned)</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>App = P1 (chinese-roberta-wwm-ext) + P2 (bge-small-zh-v1.5, w=3) + plating. Deployed P1+lexicon hand-test: 0.852</t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" s="26" t="inlineStr">
+        <is>
+          <t>3 people | 今晚想吃清蒸的，配一個燙青菜</t>
+        </is>
+      </c>
+      <c r="O15" s="26" t="inlineStr">
         <is>
           <t>blanch, steam</t>
         </is>
       </c>
-      <c r="M49" s="7" t="n"/>
-      <c r="N49" s="7" t="n"/>
-    </row>
-    <row r="50">
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>testing samples (voice clips):</t>
-        </is>
-      </c>
-      <c r="F50" s="3">
+      <c r="P15" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q15" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Mozilla Common Voice 22 Yue (CC0)</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
         <f>COUNTA('P3 clips'!A2:A201)</f>
         <v/>
       </c>
-    </row>
-    <row r="51">
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>speakers / minutes of audio:</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>167 speakers / 15.2 min</t>
-        </is>
-      </c>
-      <c r="L51" s="1" t="inlineStr">
-        <is>
-          <t>Voice accuracy (Streamlit Cloud):</t>
-        </is>
-      </c>
-      <c r="N51" s="16">
-        <f>IF(COUNTA(N45:N49)=0,"not checked yet",COUNTIF(N45:N49,"Correct")/COUNTA(N45:N49))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="L52" s="15" t="inlineStr">
-        <is>
-          <t>Correct = after 'Turn into text' and 'Plan tonight's menu', the 'Understood' line on the Menu page shows exactly the expected tags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="48" customHeight="1">
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>clips</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>167 spk / 15.2 min</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="N16" s="26" t="inlineStr">
+        <is>
+          <t>4 people | quick stir fry with lots of veggies</t>
+        </is>
+      </c>
+      <c r="O16" s="26" t="inlineStr">
+        <is>
+          <t>more_veg, quick, stir</t>
+        </is>
+      </c>
+      <c r="P16" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q16" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Model name</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>Performance (character accuracy = 1 - character error rate)</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Run time (in sec. per clip, CPU)</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>Sentence accuracy (no error)</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>Parameters (millions)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="11" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Char accuracy</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Runtime s/clip</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>Sentence acc</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="N17" s="26" t="inlineStr">
+        <is>
+          <t>5 people | we want more meat tonight and a soup</t>
+        </is>
+      </c>
+      <c r="O17" s="26" t="inlineStr">
+        <is>
+          <t>more_veg, soup</t>
+        </is>
+      </c>
+      <c r="P17" s="36" t="inlineStr">
+        <is>
+          <t>Incorrect (tags)</t>
+        </is>
+      </c>
+      <c r="Q17" s="36" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Model 1</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>alvanlii/whisper-small-cantonese</t>
         </is>
       </c>
-      <c r="E54" s="12">
+      <c r="C18" s="30">
         <f>1-SUM('P3 clips'!E2:E201)/SUM('P3 clips'!C2:C201)</f>
         <v/>
       </c>
-      <c r="F54" s="13" t="n">
+      <c r="D18" s="27" t="n">
         <v>0.38</v>
       </c>
-      <c r="G54" s="12">
+      <c r="E18" s="30">
         <f>COUNTIF('P3 clips'!E2:E201,0)/COUNT('P3 clips'!E2:E201)</f>
         <v/>
       </c>
-      <c r="H54" s="17" t="n">
-        <v>241.7</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" s="5" t="inlineStr">
+      <c r="M18" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="N18" s="26" t="inlineStr">
+        <is>
+          <t>2 people | 落雨天想飲啖熱湯</t>
+        </is>
+      </c>
+      <c r="O18" s="26" t="inlineStr">
+        <is>
+          <t>soup</t>
+        </is>
+      </c>
+      <c r="P18" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q18" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>Model 2</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>safecantonese/whisper-base-yue-hk-mdccl</t>
         </is>
       </c>
-      <c r="E55" s="8">
+      <c r="C19" s="28">
         <f>1-SUM('P3 clips'!G2:G201)/SUM('P3 clips'!C2:C201)</f>
         <v/>
       </c>
-      <c r="F55" s="9" t="n">
+      <c r="D19" s="25" t="n">
         <v>0.16</v>
       </c>
-      <c r="G55" s="8">
+      <c r="E19" s="28">
         <f>COUNTIF('P3 clips'!G2:G201,0)/COUNT('P3 clips'!G2:G201)</f>
         <v/>
       </c>
-      <c r="H55" s="18" t="n">
-        <v>72.59999999999999</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="5" t="inlineStr">
+      <c r="M19" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="N19" s="26" t="inlineStr">
+        <is>
+          <t>4 people | 想食得有鑊氣，炒牛肉都好</t>
+        </is>
+      </c>
+      <c r="O19" s="26" t="inlineStr">
+        <is>
+          <t>stir</t>
+        </is>
+      </c>
+      <c r="P19" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q19" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Model 3</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>scottykwok/wav2vec2-large-xlsr-cantonese</t>
         </is>
       </c>
-      <c r="E56" s="8">
+      <c r="C20" s="28">
         <f>1-SUM('P3 clips'!I2:I201)/SUM('P3 clips'!C2:C201)</f>
         <v/>
       </c>
-      <c r="F56" s="9" t="n">
+      <c r="D20" s="25" t="n">
         <v>0.1</v>
       </c>
-      <c r="G56" s="8">
+      <c r="E20" s="28">
         <f>COUNTIF('P3 clips'!I2:I201,0)/COUNT('P3 clips'!I2:I201)</f>
         <v/>
       </c>
-      <c r="H56" s="18" t="n">
-        <v>319.1</v>
-      </c>
-    </row>
-    <row r="57" ht="44" customHeight="1">
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>Each model runs through the app's Transcriber (16 kHz audio; Whisper decodes greedily in Chinese). Errors ignore punctuation, spaces and simplified/traditional differences. Source: notebooks/Model3_speech.ipynb; accuracy cells are formulas over sheet 'P3 clips'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="E59" s="1" t="inlineStr">
-        <is>
-          <t>Step 2b: Pick the BEST model for implementation</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>alvanlii/whisper-small-cantonese is picked: highest character accuracy; models within one standard error of the best are tied and the shortest run time wins.</t>
+      <c r="M20" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" s="26" t="inlineStr">
+        <is>
+          <t>6 people | 蒸魚，炒菜，再加個湯</t>
+        </is>
+      </c>
+      <c r="O20" s="26" t="inlineStr">
+        <is>
+          <t>soup, steam, stir</t>
+        </is>
+      </c>
+      <c r="P20" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q20" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Char acc = 1−CER. Params (M): 241.7 / 72.6 / 319.1. Source: Model3_speech.ipynb</t>
+        </is>
+      </c>
+      <c r="M21" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="N21" s="26" t="inlineStr">
+        <is>
+          <t>3 people | 十五分鐘煮好，灼個菜蒸條魚</t>
+        </is>
+      </c>
+      <c r="O21" s="26" t="inlineStr">
+        <is>
+          <t>blanch, quick, steam</t>
+        </is>
+      </c>
+      <c r="P21" s="36" t="inlineStr">
+        <is>
+          <t>Incorrect (methods on menu)</t>
+        </is>
+      </c>
+      <c r="Q21" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>PICK</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>alvanlii/whisper-small-cantonese (highest char accuracy)</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="M22" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" s="26" t="inlineStr">
+        <is>
+          <t>4 people | 多菜少肉，唔好甜  [chips: quick]</t>
+        </is>
+      </c>
+      <c r="O22" s="26" t="inlineStr">
+        <is>
+          <t>less_sweet, more_veg, quick</t>
+        </is>
+      </c>
+      <c r="P22" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q22" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="M23" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="N23" s="26" t="inlineStr">
+        <is>
+          <t>2 people | 隨便啦  [chips: blanch]</t>
+        </is>
+      </c>
+      <c r="O23" s="26" t="inlineStr">
+        <is>
+          <t>blanch</t>
+        </is>
+      </c>
+      <c r="P23" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q23" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="M24" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="N24" s="26" t="inlineStr">
+        <is>
+          <t>5 people | 長輩血糖高，不要甜的</t>
+        </is>
+      </c>
+      <c r="O24" s="26" t="inlineStr">
+        <is>
+          <t>less_sweet</t>
+        </is>
+      </c>
+      <c r="P24" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q24" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="M25" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="N25" s="26" t="inlineStr">
+        <is>
+          <t>4 people | 雪櫃有雞胸同菠菜</t>
+        </is>
+      </c>
+      <c r="O25" s="26" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="P25" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="Q25" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="O26" s="37" t="inlineStr">
+        <is>
+          <t>Notebook:</t>
+        </is>
+      </c>
+      <c r="P26" s="37">
+        <f>COUNTIF(P6:P25,"Correct")&amp;" / "&amp;COUNTA(P6:P25)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="38">
+        <f>COUNTIF(P6:P25,"Correct")/COUNTA(P6:P25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="O27" s="37" t="inlineStr">
+        <is>
+          <t>Cloud:</t>
+        </is>
+      </c>
+      <c r="P27" s="37">
+        <f>COUNTIF(Q6:Q25,"Correct")&amp;" / "&amp;COUNTA(Q6:Q25)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="38">
+        <f>IF(COUNTA(Q6:Q25)=0,"—",COUNTIF(Q6:Q25,"Correct")/COUNTA(Q6:Q25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="M28" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="N28" s="21" t="inlineStr">
+        <is>
+          <t>Judgement: tags, dish count, no repeats, methods, soup, 20-min, balance. #12 tags wrong; #16 methods (notebook only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="M30" s="33" t="inlineStr">
+        <is>
+          <t>Voice-note tests (P3: alvanlii/whisper-small-cantonese on Streamlit Cloud)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="M31" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="N31" s="24" t="inlineStr">
+        <is>
+          <t>Say (Cantonese)</t>
+        </is>
+      </c>
+      <c r="O31" s="24" t="inlineStr">
+        <is>
+          <t>Expected tags</t>
+        </is>
+      </c>
+      <c r="P31" s="24" t="inlineStr">
+        <is>
+          <t>Text heard</t>
+        </is>
+      </c>
+      <c r="Q31" s="24" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="M32" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="26" t="inlineStr">
+        <is>
+          <t>今晚想食清蒸魚，唔好太甜</t>
+        </is>
+      </c>
+      <c r="O32" s="26" t="inlineStr">
+        <is>
+          <t>steam, less_sweet</t>
+        </is>
+      </c>
+      <c r="P32" s="26" t="inlineStr">
+        <is>
+          <t>今晚想食清蒸魚唔好太甜</t>
+        </is>
+      </c>
+      <c r="Q32" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="M33" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="N33" s="26" t="inlineStr">
+        <is>
+          <t>好趕時間，炒兩個餸就得</t>
+        </is>
+      </c>
+      <c r="O33" s="26" t="inlineStr">
+        <is>
+          <t>quick, stir</t>
+        </is>
+      </c>
+      <c r="P33" s="26" t="inlineStr">
+        <is>
+          <t>好趕時間炒兩個餸就得</t>
+        </is>
+      </c>
+      <c r="Q33" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="M34" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="N34" s="26" t="inlineStr">
+        <is>
+          <t>想煲個湯，多啲菜</t>
+        </is>
+      </c>
+      <c r="O34" s="26" t="inlineStr">
+        <is>
+          <t>soup, more_veg</t>
+        </is>
+      </c>
+      <c r="P34" s="26" t="inlineStr">
+        <is>
+          <t>想煲個湯多啲菜</t>
+        </is>
+      </c>
+      <c r="Q34" s="27" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="M35" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="N35" s="26" t="inlineStr">
+        <is>
+          <t>屋企三個男仔，肉要多啲</t>
+        </is>
+      </c>
+      <c r="O35" s="26" t="inlineStr">
+        <is>
+          <t>more_meat</t>
+        </is>
+      </c>
+      <c r="P35" s="26" t="inlineStr">
+        <is>
+          <t>屋企三個男仔欲要多啲</t>
+        </is>
+      </c>
+      <c r="Q35" s="36" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="M36" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="N36" s="26" t="inlineStr">
+        <is>
+          <t>灼個菜心，再蒸個水蛋</t>
+        </is>
+      </c>
+      <c r="O36" s="26" t="inlineStr">
+        <is>
+          <t>blanch, steam</t>
+        </is>
+      </c>
+      <c r="P36" s="26" t="inlineStr">
+        <is>
+          <t>搥個菜心再蒸個水蛋</t>
+        </is>
+      </c>
+      <c r="Q36" s="36" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="O37" s="37" t="inlineStr">
+        <is>
+          <t>Voice Cloud:</t>
+        </is>
+      </c>
+      <c r="P37" s="37">
+        <f>COUNTIF(Q32:Q36,"Correct")&amp;" / "&amp;COUNTA(Q32:Q36)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="38">
+        <f>IF(COUNTA(Q32:Q36)=0,"—",COUNTIF(Q32:Q36,"Correct")/COUNTA(Q32:Q36))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="M38" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="N38" s="21" t="inlineStr">
+        <is>
+          <t>Correct = Understood tags match expected after Turn into text + Plan. #4 ASR「欲要」; #5「搥」.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D57:H57"/>
-    <mergeCell ref="L40:N40"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="L52:N52"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>